<commit_message>
Add slash commands, clean data, fix negative net tuition clip, regenerate outputs
Co-Authored-By: Claude Opus 4.7 (1M context) <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/program_summary_output.xlsx
+++ b/program_summary_output.xlsx
@@ -1,13 +1,13 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <workbookProtection/>
   <bookViews>
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Sheet1" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet name="Sheet1" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -17,16 +17,13 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="0"/>
-  <fonts count="2">
+  <fonts count="1">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
       <color theme="1"/>
       <sz val="11"/>
       <scheme val="minor"/>
-    </font>
-    <font>
-      <b val="1"/>
     </font>
   </fonts>
   <fills count="2">
@@ -37,7 +34,7 @@
       <patternFill patternType="gray125"/>
     </fill>
   </fills>
-  <borders count="2">
+  <borders count="1">
     <border>
       <left/>
       <right/>
@@ -45,21 +42,12 @@
       <bottom/>
       <diagonal/>
     </border>
-    <border>
-      <left style="thin"/>
-      <right style="thin"/>
-      <top style="thin"/>
-      <bottom style="thin"/>
-    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="2">
+  <cellXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="top"/>
-    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -425,53 +413,63 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I12"/>
+  <dimension ref="A1:K11"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
-      <c r="A1" s="1" t="inlineStr">
+      <c r="A1" t="inlineStr">
         <is>
           <t>program</t>
         </is>
       </c>
-      <c r="B1" s="1" t="inlineStr">
+      <c r="B1" t="inlineStr">
         <is>
           <t>students</t>
         </is>
       </c>
-      <c r="C1" s="1" t="inlineStr">
+      <c r="C1" t="inlineStr">
+        <is>
+          <t>intl_students</t>
+        </is>
+      </c>
+      <c r="D1" t="inlineStr">
         <is>
           <t>avg_tuition</t>
         </is>
       </c>
-      <c r="D1" s="1" t="inlineStr">
+      <c r="E1" t="inlineStr">
         <is>
           <t>avg_scholarship</t>
         </is>
       </c>
-      <c r="E1" s="1" t="inlineStr">
+      <c r="F1" t="inlineStr">
         <is>
           <t>avg_net_tuition</t>
         </is>
       </c>
-      <c r="F1" s="1" t="inlineStr">
+      <c r="G1" t="inlineStr">
         <is>
           <t>total_gross_tuition</t>
         </is>
       </c>
-      <c r="G1" s="1" t="inlineStr">
+      <c r="H1" t="inlineStr">
         <is>
           <t>total_scholarship</t>
         </is>
       </c>
-      <c r="H1" s="1" t="inlineStr">
+      <c r="I1" t="inlineStr">
         <is>
           <t>total_net_tuition</t>
         </is>
       </c>
-      <c r="I1" s="1" t="inlineStr">
+      <c r="J1" t="inlineStr">
         <is>
           <t>discount_rate</t>
+        </is>
+      </c>
+      <c r="K1" t="inlineStr">
+        <is>
+          <t>intl_pct</t>
         </is>
       </c>
     </row>
@@ -485,25 +483,31 @@
         <v>135</v>
       </c>
       <c r="C2" t="n">
+        <v>39</v>
+      </c>
+      <c r="D2" t="n">
         <v>108230.9929078014</v>
       </c>
-      <c r="D2" t="n">
+      <c r="E2" t="n">
         <v>59519.39007092199</v>
       </c>
-      <c r="E2" t="n">
+      <c r="F2" t="n">
         <v>48711.60283687944</v>
       </c>
-      <c r="F2" t="n">
+      <c r="G2" t="n">
         <v>15260570</v>
       </c>
-      <c r="G2" t="n">
+      <c r="H2" t="n">
         <v>8392234</v>
       </c>
-      <c r="H2" t="n">
+      <c r="I2" t="n">
         <v>6868336</v>
       </c>
-      <c r="I2" t="n">
+      <c r="J2" t="n">
         <v>0.5499292621442057</v>
+      </c>
+      <c r="K2" t="n">
+        <v>0.2888888888888889</v>
       </c>
     </row>
     <row r="3">
@@ -516,25 +520,31 @@
         <v>154</v>
       </c>
       <c r="C3" t="n">
+        <v>133</v>
+      </c>
+      <c r="D3" t="n">
         <v>65700.8909090909</v>
       </c>
-      <c r="D3" t="n">
+      <c r="E3" t="n">
         <v>32250.41948051948</v>
       </c>
-      <c r="E3" t="n">
-        <v>33450.47142857143</v>
-      </c>
       <c r="F3" t="n">
+        <v>33479.88051948052</v>
+      </c>
+      <c r="G3" t="n">
         <v>10117937.2</v>
       </c>
-      <c r="G3" t="n">
+      <c r="H3" t="n">
         <v>4966564.6</v>
       </c>
-      <c r="H3" t="n">
-        <v>5151372.6</v>
-      </c>
       <c r="I3" t="n">
+        <v>5155901.6</v>
+      </c>
+      <c r="J3" t="n">
         <v>0.4908673084074884</v>
+      </c>
+      <c r="K3" t="n">
+        <v>0.8636363636363636</v>
       </c>
     </row>
     <row r="4">
@@ -547,25 +557,31 @@
         <v>68</v>
       </c>
       <c r="C4" t="n">
+        <v>0</v>
+      </c>
+      <c r="D4" t="n">
         <v>53545.27058823529</v>
       </c>
-      <c r="D4" t="n">
+      <c r="E4" t="n">
         <v>5124.661764705882</v>
       </c>
-      <c r="E4" t="n">
+      <c r="F4" t="n">
         <v>48420.60882352941</v>
       </c>
-      <c r="F4" t="n">
+      <c r="G4" t="n">
         <v>3641078.4</v>
       </c>
-      <c r="G4" t="n">
+      <c r="H4" t="n">
         <v>348477</v>
       </c>
-      <c r="H4" t="n">
+      <c r="I4" t="n">
         <v>3292601.4</v>
       </c>
-      <c r="I4" t="n">
+      <c r="J4" t="n">
         <v>0.09570708502184408</v>
+      </c>
+      <c r="K4" t="n">
+        <v>0</v>
       </c>
     </row>
     <row r="5">
@@ -578,25 +594,31 @@
         <v>28</v>
       </c>
       <c r="C5" t="n">
+        <v>4</v>
+      </c>
+      <c r="D5" t="n">
         <v>61501.07142857143</v>
       </c>
-      <c r="D5" t="n">
+      <c r="E5" t="n">
         <v>15930.85714285714</v>
       </c>
-      <c r="E5" t="n">
+      <c r="F5" t="n">
         <v>45570.21428571428</v>
       </c>
-      <c r="F5" t="n">
+      <c r="G5" t="n">
         <v>1722030</v>
       </c>
-      <c r="G5" t="n">
+      <c r="H5" t="n">
         <v>446064</v>
       </c>
-      <c r="H5" t="n">
+      <c r="I5" t="n">
         <v>1275966</v>
       </c>
-      <c r="I5" t="n">
+      <c r="J5" t="n">
         <v>0.2590338147419035</v>
+      </c>
+      <c r="K5" t="n">
+        <v>0.1428571428571428</v>
       </c>
     </row>
     <row r="6">
@@ -609,25 +631,31 @@
         <v>27</v>
       </c>
       <c r="C6" t="n">
+        <v>2</v>
+      </c>
+      <c r="D6" t="n">
         <v>45221.7037037037</v>
       </c>
-      <c r="D6" t="n">
+      <c r="E6" t="n">
         <v>7199</v>
       </c>
-      <c r="E6" t="n">
+      <c r="F6" t="n">
         <v>38022.7037037037</v>
       </c>
-      <c r="F6" t="n">
+      <c r="G6" t="n">
         <v>1220986</v>
       </c>
-      <c r="G6" t="n">
+      <c r="H6" t="n">
         <v>194373</v>
       </c>
-      <c r="H6" t="n">
+      <c r="I6" t="n">
         <v>1026613</v>
       </c>
-      <c r="I6" t="n">
+      <c r="J6" t="n">
         <v>0.1591934715058158</v>
+      </c>
+      <c r="K6" t="n">
+        <v>0.07407407407407407</v>
       </c>
     </row>
     <row r="7">
@@ -640,25 +668,31 @@
         <v>19</v>
       </c>
       <c r="C7" t="n">
+        <v>8</v>
+      </c>
+      <c r="D7" t="n">
         <v>57857.68421052631</v>
       </c>
-      <c r="D7" t="n">
+      <c r="E7" t="n">
         <v>23709.57894736842</v>
       </c>
-      <c r="E7" t="n">
+      <c r="F7" t="n">
         <v>34148.10526315789</v>
       </c>
-      <c r="F7" t="n">
+      <c r="G7" t="n">
         <v>1099296</v>
       </c>
-      <c r="G7" t="n">
+      <c r="H7" t="n">
         <v>450482</v>
       </c>
-      <c r="H7" t="n">
+      <c r="I7" t="n">
         <v>648814</v>
       </c>
-      <c r="I7" t="n">
+      <c r="J7" t="n">
         <v>0.4097913573778127</v>
+      </c>
+      <c r="K7" t="n">
+        <v>0.4210526315789473</v>
       </c>
     </row>
     <row r="8">
@@ -671,56 +705,68 @@
         <v>11</v>
       </c>
       <c r="C8" t="n">
+        <v>0</v>
+      </c>
+      <c r="D8" t="n">
         <v>56451.63636363636</v>
       </c>
-      <c r="D8" t="n">
-        <v>0</v>
-      </c>
       <c r="E8" t="n">
+        <v>0</v>
+      </c>
+      <c r="F8" t="n">
         <v>56451.63636363636</v>
       </c>
-      <c r="F8" t="n">
+      <c r="G8" t="n">
         <v>620968</v>
       </c>
-      <c r="G8" t="n">
-        <v>0</v>
-      </c>
       <c r="H8" t="n">
+        <v>0</v>
+      </c>
+      <c r="I8" t="n">
         <v>620968</v>
       </c>
-      <c r="I8" t="n">
+      <c r="J8" t="n">
+        <v>0</v>
+      </c>
+      <c r="K8" t="n">
         <v>0</v>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>Economics 4+1</t>
+          <t>Economics</t>
         </is>
       </c>
       <c r="B9" t="n">
-        <v>16</v>
+        <v>18</v>
       </c>
       <c r="C9" t="n">
-        <v>46712.5</v>
+        <v>5</v>
       </c>
       <c r="D9" t="n">
-        <v>18566.25</v>
+        <v>45588.88888888889</v>
       </c>
       <c r="E9" t="n">
-        <v>28146.25</v>
+        <v>16910</v>
       </c>
       <c r="F9" t="n">
-        <v>747400</v>
+        <v>28678.88888888889</v>
       </c>
       <c r="G9" t="n">
-        <v>297060</v>
+        <v>820600</v>
       </c>
       <c r="H9" t="n">
-        <v>450340</v>
+        <v>304380</v>
       </c>
       <c r="I9" t="n">
-        <v>0.3974578538934975</v>
+        <v>516220</v>
+      </c>
+      <c r="J9" t="n">
+        <v>0.3709237143553498</v>
+      </c>
+      <c r="K9" t="n">
+        <v>0.2777777777777778</v>
       </c>
     </row>
     <row r="10">
@@ -733,25 +779,31 @@
         <v>19</v>
       </c>
       <c r="C10" t="n">
+        <v>5</v>
+      </c>
+      <c r="D10" t="n">
         <v>42788.63157894737</v>
       </c>
-      <c r="D10" t="n">
+      <c r="E10" t="n">
         <v>21157.26315789474</v>
       </c>
-      <c r="E10" t="n">
+      <c r="F10" t="n">
         <v>21631.36842105263</v>
       </c>
-      <c r="F10" t="n">
+      <c r="G10" t="n">
         <v>812984</v>
       </c>
-      <c r="G10" t="n">
+      <c r="H10" t="n">
         <v>401988</v>
       </c>
-      <c r="H10" t="n">
+      <c r="I10" t="n">
         <v>410996</v>
       </c>
-      <c r="I10" t="n">
+      <c r="J10" t="n">
         <v>0.4944599155702941</v>
+      </c>
+      <c r="K10" t="n">
+        <v>0.2631578947368421</v>
       </c>
     </row>
     <row r="11">
@@ -764,56 +816,31 @@
         <v>8</v>
       </c>
       <c r="C11" t="n">
+        <v>0</v>
+      </c>
+      <c r="D11" t="n">
         <v>48800</v>
       </c>
-      <c r="D11" t="n">
-        <v>0</v>
-      </c>
       <c r="E11" t="n">
+        <v>0</v>
+      </c>
+      <c r="F11" t="n">
         <v>48800</v>
       </c>
-      <c r="F11" t="n">
+      <c r="G11" t="n">
         <v>390400</v>
       </c>
-      <c r="G11" t="n">
-        <v>0</v>
-      </c>
       <c r="H11" t="n">
+        <v>0</v>
+      </c>
+      <c r="I11" t="n">
         <v>390400</v>
       </c>
-      <c r="I11" t="n">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="12">
-      <c r="A12" t="inlineStr">
-        <is>
-          <t>Economics</t>
-        </is>
-      </c>
-      <c r="B12" t="n">
-        <v>2</v>
-      </c>
-      <c r="C12" t="n">
-        <v>36600</v>
-      </c>
-      <c r="D12" t="n">
-        <v>3660</v>
-      </c>
-      <c r="E12" t="n">
-        <v>32940</v>
-      </c>
-      <c r="F12" t="n">
-        <v>73200</v>
-      </c>
-      <c r="G12" t="n">
-        <v>7320</v>
-      </c>
-      <c r="H12" t="n">
-        <v>65880</v>
-      </c>
-      <c r="I12" t="n">
-        <v>0.1</v>
+      <c r="J11" t="n">
+        <v>0</v>
+      </c>
+      <c r="K11" t="n">
+        <v>0</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Add academic-year dimension and program-specific annualization
- Decode PeopleSoft term codes to academic year; aggregate at (ID, plan, AY)
- Add terms_per_year lookup (Info Sheet + empirical); fix peer annualization
- Emit student_program_year_output.xlsx for cohort-year analysis
- Fix cell 2 to persist intl columns in on-disk outputs
- CLAUDE.md: note Multi-Year file is byte-identical duplicate; document AY decoding and terms-per-year table

Co-Authored-By: Claude Opus 4.7 (1M context) <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/program_summary_output.xlsx
+++ b/program_summary_output.xlsx
@@ -504,10 +504,10 @@
         <v>6868336</v>
       </c>
       <c r="J2" t="n">
-        <v>0.5499292621442057</v>
+        <v>54.99292621442057</v>
       </c>
       <c r="K2" t="n">
-        <v>0.2888888888888889</v>
+        <v>28.88888888888889</v>
       </c>
     </row>
     <row r="3">
@@ -541,10 +541,10 @@
         <v>5155901.6</v>
       </c>
       <c r="J3" t="n">
-        <v>0.4908673084074884</v>
+        <v>49.08673084074884</v>
       </c>
       <c r="K3" t="n">
-        <v>0.8636363636363636</v>
+        <v>86.36363636363636</v>
       </c>
     </row>
     <row r="4">
@@ -578,7 +578,7 @@
         <v>3292601.4</v>
       </c>
       <c r="J4" t="n">
-        <v>0.09570708502184408</v>
+        <v>9.570708502184408</v>
       </c>
       <c r="K4" t="n">
         <v>0</v>
@@ -615,10 +615,10 @@
         <v>1275966</v>
       </c>
       <c r="J5" t="n">
-        <v>0.2590338147419035</v>
+        <v>25.90338147419035</v>
       </c>
       <c r="K5" t="n">
-        <v>0.1428571428571428</v>
+        <v>14.28571428571428</v>
       </c>
     </row>
     <row r="6">
@@ -652,10 +652,10 @@
         <v>1026613</v>
       </c>
       <c r="J6" t="n">
-        <v>0.1591934715058158</v>
+        <v>15.91934715058158</v>
       </c>
       <c r="K6" t="n">
-        <v>0.07407407407407407</v>
+        <v>7.407407407407407</v>
       </c>
     </row>
     <row r="7">
@@ -689,10 +689,10 @@
         <v>648814</v>
       </c>
       <c r="J7" t="n">
-        <v>0.4097913573778127</v>
+        <v>40.97913573778127</v>
       </c>
       <c r="K7" t="n">
-        <v>0.4210526315789473</v>
+        <v>42.10526315789473</v>
       </c>
     </row>
     <row r="8">
@@ -748,25 +748,25 @@
         <v>45588.88888888889</v>
       </c>
       <c r="E9" t="n">
-        <v>16910</v>
+        <v>15610</v>
       </c>
       <c r="F9" t="n">
-        <v>28678.88888888889</v>
+        <v>29978.88888888889</v>
       </c>
       <c r="G9" t="n">
         <v>820600</v>
       </c>
       <c r="H9" t="n">
-        <v>304380</v>
+        <v>280980</v>
       </c>
       <c r="I9" t="n">
-        <v>516220</v>
+        <v>539620</v>
       </c>
       <c r="J9" t="n">
-        <v>0.3709237143553498</v>
+        <v>34.24079941506215</v>
       </c>
       <c r="K9" t="n">
-        <v>0.2777777777777778</v>
+        <v>27.77777777777778</v>
       </c>
     </row>
     <row r="10">
@@ -800,10 +800,10 @@
         <v>410996</v>
       </c>
       <c r="J10" t="n">
-        <v>0.4944599155702941</v>
+        <v>49.44599155702941</v>
       </c>
       <c r="K10" t="n">
-        <v>0.2631578947368421</v>
+        <v>26.31578947368421</v>
       </c>
     </row>
     <row r="11">

</xml_diff>

<commit_message>
Add df_pricing filter for partial-term students in pricing charts
Partial-term rows (total tuition < $20k) were pulling down avg gross/net
tuition and compressing discount rates for the typical full-load student.
Introduce df_pricing and a pricing_summary tab used only for discount
rate, gross-vs-net, and peer benchmark charts. Enrollment, intl mix, and
trend charts still run on the full population.

Co-Authored-By: Claude Opus 4.7 (1M context) <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/program_summary_output.xlsx
+++ b/program_summary_output.xlsx
@@ -1,13 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <workbookProtection/>
   <bookViews>
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet name="Sheet1" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="program_summary" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="pricing_summary" sheetId="2" state="visible" r:id="rId2"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -846,4 +847,375 @@
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:I11"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <sheetData>
+    <row r="1">
+      <c r="A1" t="inlineStr">
+        <is>
+          <t>program</t>
+        </is>
+      </c>
+      <c r="B1" t="inlineStr">
+        <is>
+          <t>students</t>
+        </is>
+      </c>
+      <c r="C1" t="inlineStr">
+        <is>
+          <t>avg_tuition</t>
+        </is>
+      </c>
+      <c r="D1" t="inlineStr">
+        <is>
+          <t>avg_scholarship</t>
+        </is>
+      </c>
+      <c r="E1" t="inlineStr">
+        <is>
+          <t>avg_net_tuition</t>
+        </is>
+      </c>
+      <c r="F1" t="inlineStr">
+        <is>
+          <t>total_gross_tuition</t>
+        </is>
+      </c>
+      <c r="G1" t="inlineStr">
+        <is>
+          <t>total_scholarship</t>
+        </is>
+      </c>
+      <c r="H1" t="inlineStr">
+        <is>
+          <t>total_net_tuition</t>
+        </is>
+      </c>
+      <c r="I1" t="inlineStr">
+        <is>
+          <t>discount_rate</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="inlineStr">
+        <is>
+          <t>MDP</t>
+        </is>
+      </c>
+      <c r="B2" t="n">
+        <v>135</v>
+      </c>
+      <c r="C2" t="n">
+        <v>108230.9929078014</v>
+      </c>
+      <c r="D2" t="n">
+        <v>59519.39007092199</v>
+      </c>
+      <c r="E2" t="n">
+        <v>48711.60283687944</v>
+      </c>
+      <c r="F2" t="n">
+        <v>15260570</v>
+      </c>
+      <c r="G2" t="n">
+        <v>8392234</v>
+      </c>
+      <c r="H2" t="n">
+        <v>6868336</v>
+      </c>
+      <c r="I2" t="n">
+        <v>54.99292621442057</v>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="inlineStr">
+        <is>
+          <t>Computer Science</t>
+        </is>
+      </c>
+      <c r="B3" t="n">
+        <v>150</v>
+      </c>
+      <c r="C3" t="n">
+        <v>67143.23466666666</v>
+      </c>
+      <c r="D3" t="n">
+        <v>33020.61733333333</v>
+      </c>
+      <c r="E3" t="n">
+        <v>34152.81066666666</v>
+      </c>
+      <c r="F3" t="n">
+        <v>10071485.2</v>
+      </c>
+      <c r="G3" t="n">
+        <v>4953092.6</v>
+      </c>
+      <c r="H3" t="n">
+        <v>5122921.6</v>
+      </c>
+      <c r="I3" t="n">
+        <v>49.1793663163006</v>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="inlineStr">
+        <is>
+          <t>Bioethics</t>
+        </is>
+      </c>
+      <c r="B4" t="n">
+        <v>62</v>
+      </c>
+      <c r="C4" t="n">
+        <v>57343.24838709677</v>
+      </c>
+      <c r="D4" t="n">
+        <v>5467.548387096775</v>
+      </c>
+      <c r="E4" t="n">
+        <v>51875.7</v>
+      </c>
+      <c r="F4" t="n">
+        <v>3555281.4</v>
+      </c>
+      <c r="G4" t="n">
+        <v>338988</v>
+      </c>
+      <c r="H4" t="n">
+        <v>3216293.4</v>
+      </c>
+      <c r="I4" t="n">
+        <v>9.534772690566772</v>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>Cancer Biology 4+1</t>
+        </is>
+      </c>
+      <c r="B5" t="n">
+        <v>28</v>
+      </c>
+      <c r="C5" t="n">
+        <v>61501.07142857143</v>
+      </c>
+      <c r="D5" t="n">
+        <v>15930.85714285714</v>
+      </c>
+      <c r="E5" t="n">
+        <v>45570.21428571428</v>
+      </c>
+      <c r="F5" t="n">
+        <v>1722030</v>
+      </c>
+      <c r="G5" t="n">
+        <v>446064</v>
+      </c>
+      <c r="H5" t="n">
+        <v>1275966</v>
+      </c>
+      <c r="I5" t="n">
+        <v>25.90338147419035</v>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="inlineStr">
+        <is>
+          <t>Bioethics 4+1</t>
+        </is>
+      </c>
+      <c r="B6" t="n">
+        <v>26</v>
+      </c>
+      <c r="C6" t="n">
+        <v>46241</v>
+      </c>
+      <c r="D6" t="n">
+        <v>7385.884615384615</v>
+      </c>
+      <c r="E6" t="n">
+        <v>38855.11538461538</v>
+      </c>
+      <c r="F6" t="n">
+        <v>1202266</v>
+      </c>
+      <c r="G6" t="n">
+        <v>192033</v>
+      </c>
+      <c r="H6" t="n">
+        <v>1010233</v>
+      </c>
+      <c r="I6" t="n">
+        <v>15.97258842885019</v>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="inlineStr">
+        <is>
+          <t>Math</t>
+        </is>
+      </c>
+      <c r="B7" t="n">
+        <v>19</v>
+      </c>
+      <c r="C7" t="n">
+        <v>57857.68421052631</v>
+      </c>
+      <c r="D7" t="n">
+        <v>23709.57894736842</v>
+      </c>
+      <c r="E7" t="n">
+        <v>34148.10526315789</v>
+      </c>
+      <c r="F7" t="n">
+        <v>1099296</v>
+      </c>
+      <c r="G7" t="n">
+        <v>450482</v>
+      </c>
+      <c r="H7" t="n">
+        <v>648814</v>
+      </c>
+      <c r="I7" t="n">
+        <v>40.97913573778127</v>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="inlineStr">
+        <is>
+          <t>Data Science</t>
+        </is>
+      </c>
+      <c r="B8" t="n">
+        <v>11</v>
+      </c>
+      <c r="C8" t="n">
+        <v>56451.63636363636</v>
+      </c>
+      <c r="D8" t="n">
+        <v>0</v>
+      </c>
+      <c r="E8" t="n">
+        <v>56451.63636363636</v>
+      </c>
+      <c r="F8" t="n">
+        <v>620968</v>
+      </c>
+      <c r="G8" t="n">
+        <v>0</v>
+      </c>
+      <c r="H8" t="n">
+        <v>620968</v>
+      </c>
+      <c r="I8" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="inlineStr">
+        <is>
+          <t>Economics</t>
+        </is>
+      </c>
+      <c r="B9" t="n">
+        <v>18</v>
+      </c>
+      <c r="C9" t="n">
+        <v>45588.88888888889</v>
+      </c>
+      <c r="D9" t="n">
+        <v>15610</v>
+      </c>
+      <c r="E9" t="n">
+        <v>29978.88888888889</v>
+      </c>
+      <c r="F9" t="n">
+        <v>820600</v>
+      </c>
+      <c r="G9" t="n">
+        <v>280980</v>
+      </c>
+      <c r="H9" t="n">
+        <v>539620</v>
+      </c>
+      <c r="I9" t="n">
+        <v>34.24079941506215</v>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="inlineStr">
+        <is>
+          <t>Computer Science 4+1</t>
+        </is>
+      </c>
+      <c r="B10" t="n">
+        <v>19</v>
+      </c>
+      <c r="C10" t="n">
+        <v>42788.63157894737</v>
+      </c>
+      <c r="D10" t="n">
+        <v>21157.26315789474</v>
+      </c>
+      <c r="E10" t="n">
+        <v>21631.36842105263</v>
+      </c>
+      <c r="F10" t="n">
+        <v>812984</v>
+      </c>
+      <c r="G10" t="n">
+        <v>401988</v>
+      </c>
+      <c r="H10" t="n">
+        <v>410996</v>
+      </c>
+      <c r="I10" t="n">
+        <v>49.44599155702941</v>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="inlineStr">
+        <is>
+          <t>MBID</t>
+        </is>
+      </c>
+      <c r="B11" t="n">
+        <v>8</v>
+      </c>
+      <c r="C11" t="n">
+        <v>48800</v>
+      </c>
+      <c r="D11" t="n">
+        <v>0</v>
+      </c>
+      <c r="E11" t="n">
+        <v>48800</v>
+      </c>
+      <c r="F11" t="n">
+        <v>390400</v>
+      </c>
+      <c r="G11" t="n">
+        <v>0</v>
+      </c>
+      <c r="H11" t="n">
+        <v>390400</v>
+      </c>
+      <c r="I11" t="n">
+        <v>0</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
 </file>
</xml_diff>